<commit_message>
ACDR2026: reception 1007 materials, movement table times, 10/9 afternoon drafts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011xF77D95cDW5CT1JUxj7vg
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_9_Oct_v2_96.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_9_Oct_v2_96.xlsx
@@ -6360,7 +6360,7 @@
       </c>
       <c r="I5" s="27" t="inlineStr">
         <is>
-          <t>16:00設営→18:50 VIP 控え（サロン）→19:00-20:30 大使公邸レセプション（GOH: Commissioner Eric Yap）</t>
+          <t>16:00設営→18:20 大使表敬（小サロン）→19:00-20:45 大使公邸レセプション（GOH: Commissioner Eric Yap、21:00撤収）</t>
         </is>
       </c>
       <c r="J5" s="27" t="inlineStr">
@@ -7908,7 +7908,7 @@
       <c r="Y4" s="95" t="n"/>
       <c r="Z4" s="153" t="inlineStr">
         <is>
-          <t>19:00 開会（ADRC MC）／19:03 大使挨拶／19:06 GOH（Commissioner Eric Yap）挨拶／19:09 林室長乾杯／19:12-19:17 集合写真（大サロン、撮影は荒木田）／20:15 仙台市（APMCDRR2027）／20:30 閉会（Sylvia 案は 20:45、要統一）</t>
+          <t>18:20-18:40 大使表敬（小サロン）／19:00 開会（ADRC MC）／19:03 大使挨拶／19:07 GOH（Commissioner Eric Yap）挨拶／19:10 林室長乾杯／19:12-19:17 集合写真（大サロン、撮影は荒木田）／20:30 仙台市副市長の中締め（APMCDRR2027）／20:45 終了アナウンス／21:00 完全撤収（児玉さん 10/9 送付の公邸資料 1007 版。同資料 p.1 は集合写真の時刻を「検討中」、p.7 は 19:12-19:17）</t>
         </is>
       </c>
       <c r="AA4" s="94" t="n"/>
@@ -8586,7 +8586,8 @@
 (1) 19:00-21:00に受付(名札セット配布100-120名)・MC・VIP対応・写真・バス誘導(Dorsett→公邸)が同時発生。受付2名(藤中・田中)＋吉田で名札配布、藤本が写真。
 (2) 27日午前は全員で会場下見のため、Dorsettは藤中・田中のみ。午後はDorsett到着対応と公邸設営準備が並行、荒木田・池田は機材、児玉と吉田は公邸に張り付く。それ以外は到着対応補助。
 (3) 開始が19:00（8/26版アジェンダ）に後ろ倒しになったため、Dorsett→公邸の送迎バス出発（従来想定17:30〜18:30）と撤収時刻をCOSEMと再確認する必要がある。　(4)【9/25】役員（三浦・北本・宮木）は27日午前に会場を短時間見た後、大使館へ表敬（荒木田が足立氏と調整）。会場の前日設営が可能な時刻が判明したら、公邸レセプションを外れて設営に残る者を決める。
-(5)【10/8】GOH は Commissioner Eric Yap（児玉→Sylvia 10/8）。集合写真は 19:12-19:17 に大サロンで、撮影は ADRC 職員のみ（公邸資料 asof8Oct）。撮影は荒木田（10/9）。SCDF の車両番号・運転手名の事前登録を Sylvia に依頼済み。</t>
+(5)【10/8】GOH は Commissioner Eric Yap（児玉→Sylvia 10/8）。集合写真は 19:12-19:17 に大サロンで、撮影は ADRC 職員のみ（公邸資料 asof8Oct）。撮影は荒木田（10/9）。SCDF の車両番号・運転手名の事前登録を Sylvia に依頼済み。
+(6)【10/9】公邸資料 1007 版（児玉 10/9 送付）: 閉会は 20:30 仙台市中締め→20:45 終了アナウンス→21:00 撤収。18:20 大使表敬（三浦・北本・宮木、バックシート児玉）。スタッフ案では広報（写真）が塩見・森川となっており、集合写真の撮影者（荒木田）と食い違う【児玉さんに確認】。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ACDR2026: restore cached formula values (staff names) in movement table v2_96
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011xF77D95cDW5CT1JUxj7vg
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_9_Oct_v2_96.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_9_Oct_v2_96.xlsx
@@ -2595,7 +2595,7 @@
       </c>
       <c r="E26" s="10">
         <f>COUNTIF(E5:E23,"確定*")</f>
-        <v/>
+        <v>13</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="107">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="E27" s="10">
         <f>COUNTIF(E5:E23,"見込*")+COUNTIF(E5:E23,"候補*")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="107">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="E28" s="10">
         <f>COUNTIF(E5:E23,"未定*")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="107">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="E30" s="10">
         <f>E26+COUNTIF(E5:E23,"見込*")-E29</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="E31" s="12">
         <f>COUNTIF(E5:E23,"国内サポート（確定）")</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="107">
@@ -6407,9 +6407,9 @@
       <c r="S5" s="25" t="n"/>
     </row>
     <row r="6" ht="39.75" customHeight="1" s="107">
-      <c r="A6" s="28">
+      <c r="A6" s="28" t="str">
         <f>人員一覧・判定!B5</f>
-        <v/>
+        <v>三浦 房紀</v>
       </c>
       <c r="B6" s="29" t="n"/>
       <c r="C6" s="29" t="n"/>
@@ -6475,9 +6475,9 @@
       <c r="S6" s="29" t="n"/>
     </row>
     <row r="7" ht="39.75" customHeight="1" s="107">
-      <c r="A7" s="28">
+      <c r="A7" s="28" t="str">
         <f>人員一覧・判定!B6</f>
-        <v/>
+        <v>北本 政行</v>
       </c>
       <c r="B7" s="29" t="n"/>
       <c r="C7" s="29" t="n"/>
@@ -6543,9 +6543,9 @@
       <c r="S7" s="29" t="n"/>
     </row>
     <row r="8" ht="39.75" customHeight="1" s="107">
-      <c r="A8" s="28">
+      <c r="A8" s="28" t="str">
         <f>人員一覧・判定!B7</f>
-        <v/>
+        <v>宮木 一寛</v>
       </c>
       <c r="B8" s="29" t="n"/>
       <c r="C8" s="29" t="n"/>
@@ -6615,9 +6615,9 @@
       <c r="S8" s="29" t="n"/>
     </row>
     <row r="9" ht="39.75" customHeight="1" s="107">
-      <c r="A9" s="28">
+      <c r="A9" s="28" t="str">
         <f>人員一覧・判定!B8</f>
-        <v/>
+        <v>児玉 美樹</v>
       </c>
       <c r="B9" s="29" t="n"/>
       <c r="C9" s="29" t="n"/>
@@ -6687,9 +6687,9 @@
       <c r="S9" s="29" t="n"/>
     </row>
     <row r="10" ht="39.75" customHeight="1" s="107">
-      <c r="A10" s="40">
+      <c r="A10" s="40" t="str">
         <f>人員一覧・判定!B9</f>
-        <v/>
+        <v>荒木田 勝</v>
       </c>
       <c r="B10" s="29" t="n"/>
       <c r="C10" s="29" t="n"/>
@@ -6755,9 +6755,9 @@
       <c r="S10" s="29" t="n"/>
     </row>
     <row r="11" ht="39.75" customHeight="1" s="107">
-      <c r="A11" s="40">
+      <c r="A11" s="40" t="str">
         <f>人員一覧・判定!B10</f>
-        <v/>
+        <v>吉田 真紀</v>
       </c>
       <c r="B11" s="29" t="n"/>
       <c r="C11" s="29" t="n"/>
@@ -6831,9 +6831,9 @@
       <c r="S11" s="29" t="n"/>
     </row>
     <row r="12" ht="39.75" customHeight="1" s="107">
-      <c r="A12" s="40">
+      <c r="A12" s="40" t="str">
         <f>人員一覧・判定!B11</f>
-        <v/>
+        <v>藤中 純子</v>
       </c>
       <c r="B12" s="29" t="n"/>
       <c r="C12" s="29" t="n"/>
@@ -6919,9 +6919,9 @@
       </c>
     </row>
     <row r="13" ht="39.75" customHeight="1" s="107">
-      <c r="A13" s="40">
+      <c r="A13" s="40" t="str">
         <f>人員一覧・判定!B12</f>
-        <v/>
+        <v>田中 智美</v>
       </c>
       <c r="B13" s="29" t="n"/>
       <c r="C13" s="29" t="n"/>
@@ -7007,9 +7007,9 @@
       </c>
     </row>
     <row r="14" ht="39.75" customHeight="1" s="107">
-      <c r="A14" s="40">
+      <c r="A14" s="40" t="str">
         <f>人員一覧・判定!B13</f>
-        <v/>
+        <v>池田　誠</v>
       </c>
       <c r="B14" s="29" t="n"/>
       <c r="C14" s="29" t="n"/>
@@ -7075,9 +7075,9 @@
       <c r="S14" s="29" t="n"/>
     </row>
     <row r="15" ht="39.75" customHeight="1" s="107">
-      <c r="A15" s="40">
+      <c r="A15" s="40" t="str">
         <f>人員一覧・判定!C14</f>
-        <v/>
+        <v>Gerald Ejem Potutan</v>
       </c>
       <c r="B15" s="29" t="n"/>
       <c r="C15" s="29" t="n"/>
@@ -7143,9 +7143,9 @@
       <c r="S15" s="29" t="n"/>
     </row>
     <row r="16" ht="39.75" customHeight="1" s="107">
-      <c r="A16" s="40">
+      <c r="A16" s="40" t="str">
         <f>人員一覧・判定!C15</f>
-        <v/>
+        <v>Mizan Bisri</v>
       </c>
       <c r="B16" s="29" t="n"/>
       <c r="C16" s="29" t="n"/>
@@ -7211,9 +7211,9 @@
       <c r="S16" s="29" t="n"/>
     </row>
     <row r="17" ht="39.75" customHeight="1" s="107">
-      <c r="A17" s="40">
+      <c r="A17" s="40" t="str">
         <f>人員一覧・判定!B16</f>
-        <v/>
+        <v>藤本 絢子</v>
       </c>
       <c r="B17" s="29" t="n"/>
       <c r="C17" s="29" t="n"/>
@@ -7279,9 +7279,9 @@
       <c r="S17" s="29" t="n"/>
     </row>
     <row r="18" ht="39.75" customHeight="1" s="107">
-      <c r="A18" s="40">
+      <c r="A18" s="40" t="str">
         <f>人員一覧・判定!B17</f>
-        <v/>
+        <v>塩見 有美</v>
       </c>
       <c r="B18" s="29" t="n"/>
       <c r="C18" s="29" t="n"/>
@@ -7354,75 +7354,75 @@
       </c>
       <c r="B19" s="46">
         <f>COUNTA(B6:B18)-COUNTIF(B6:B18,"*未手配*")-COUNTIF(B6:B18,"*要確認*")-COUNTIF(B6:B18,"*NRT着*")-COUNTIF(B6:B18,"*HND着*")-COUNTIF(B6:B18,"*KIX着*")-COUNTIF(B6:B18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C19" s="46">
         <f>COUNTA(C6:C18)-COUNTIF(C6:C18,"*未手配*")-COUNTIF(C6:C18,"*要確認*")-COUNTIF(C6:C18,"*NRT着*")-COUNTIF(C6:C18,"*HND着*")-COUNTIF(C6:C18,"*KIX着*")-COUNTIF(C6:C18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="46">
         <f>COUNTA(D6:D18)-COUNTIF(D6:D18,"*未手配*")-COUNTIF(D6:D18,"*要確認*")-COUNTIF(D6:D18,"*NRT着*")-COUNTIF(D6:D18,"*HND着*")-COUNTIF(D6:D18,"*KIX着*")-COUNTIF(D6:D18,"*GVA着*")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="E19" s="46">
         <f>COUNTA(E6:E18)-COUNTIF(E6:E18,"*未手配*")-COUNTIF(E6:E18,"*要確認*")-COUNTIF(E6:E18,"*NRT着*")-COUNTIF(E6:E18,"*HND着*")-COUNTIF(E6:E18,"*KIX着*")-COUNTIF(E6:E18,"*GVA着*")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="F19" s="46">
         <f>COUNTA(F6:F18)-COUNTIF(F6:F18,"*未手配*")-COUNTIF(F6:F18,"*要確認*")-COUNTIF(F6:F18,"*NRT着*")-COUNTIF(F6:F18,"*HND着*")-COUNTIF(F6:F18,"*KIX着*")-COUNTIF(F6:F18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="G19" s="46">
         <f>COUNTA(G6:G18)-COUNTIF(G6:G18,"*未手配*")-COUNTIF(G6:G18,"*要確認*")-COUNTIF(G6:G18,"*NRT着*")-COUNTIF(G6:G18,"*HND着*")-COUNTIF(G6:G18,"*KIX着*")-COUNTIF(G6:G18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="H19" s="46">
         <f>COUNTA(H6:H18)-COUNTIF(H6:H18,"*未手配*")-COUNTIF(H6:H18,"*要確認*")-COUNTIF(H6:H18,"*NRT着*")-COUNTIF(H6:H18,"*HND着*")-COUNTIF(H6:H18,"*KIX着*")-COUNTIF(H6:H18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="I19" s="46">
         <f>COUNTA(I6:I18)-COUNTIF(I6:I18,"*未手配*")-COUNTIF(I6:I18,"*要確認*")-COUNTIF(I6:I18,"*NRT着*")-COUNTIF(I6:I18,"*HND着*")-COUNTIF(I6:I18,"*KIX着*")-COUNTIF(I6:I18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="J19" s="46">
         <f>COUNTA(J6:J18)-COUNTIF(J6:J18,"*未手配*")-COUNTIF(J6:J18,"*要確認*")-COUNTIF(J6:J18,"*NRT着*")-COUNTIF(J6:J18,"*HND着*")-COUNTIF(J6:J18,"*KIX着*")-COUNTIF(J6:J18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="K19" s="46">
         <f>COUNTA(K6:K18)-COUNTIF(K6:K18,"*未手配*")-COUNTIF(K6:K18,"*要確認*")-COUNTIF(K6:K18,"*NRT着*")-COUNTIF(K6:K18,"*HND着*")-COUNTIF(K6:K18,"*KIX着*")-COUNTIF(K6:K18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="L19" s="46">
         <f>COUNTA(L6:L18)-COUNTIF(L6:L18,"*未手配*")-COUNTIF(L6:L18,"*要確認*")-COUNTIF(L6:L18,"*NRT着*")-COUNTIF(L6:L18,"*HND着*")-COUNTIF(L6:L18,"*KIX着*")-COUNTIF(L6:L18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="M19" s="46">
         <f>COUNTA(M6:M18)-COUNTIF(M6:M18,"*未手配*")-COUNTIF(M6:M18,"*要確認*")-COUNTIF(M6:M18,"*NRT着*")-COUNTIF(M6:M18,"*HND着*")-COUNTIF(M6:M18,"*KIX着*")-COUNTIF(M6:M18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="N19" s="46">
         <f>COUNTA(N6:N18)-COUNTIF(N6:N18,"*未手配*")-COUNTIF(N6:N18,"*要確認*")-COUNTIF(N6:N18,"*NRT着*")-COUNTIF(N6:N18,"*HND着*")-COUNTIF(N6:N18,"*KIX着*")-COUNTIF(N6:N18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="O19" s="46">
         <f>COUNTA(O6:O18)-COUNTIF(O6:O18,"*未手配*")-COUNTIF(O6:O18,"*要確認*")-COUNTIF(O6:O18,"*NRT着*")-COUNTIF(O6:O18,"*HND着*")-COUNTIF(O6:O18,"*KIX着*")-COUNTIF(O6:O18,"*GVA着*")</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="P19" s="46">
         <f>COUNTA(P6:P18)-COUNTIF(P6:P18,"*未手配*")-COUNTIF(P6:P18,"*要確認*")-COUNTIF(P6:P18,"*NRT着*")-COUNTIF(P6:P18,"*HND着*")-COUNTIF(P6:P18,"*KIX着*")-COUNTIF(P6:P18,"*GVA着*")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="Q19" s="46">
         <f>COUNTA(Q6:Q18)-COUNTIF(Q6:Q18,"*未手配*")-COUNTIF(Q6:Q18,"*要確認*")-COUNTIF(Q6:Q18,"*NRT着*")-COUNTIF(Q6:Q18,"*HND着*")-COUNTIF(Q6:Q18,"*KIX着*")-COUNTIF(Q6:Q18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="R19" s="46">
         <f>COUNTA(R6:R18)-COUNTIF(R6:R18,"*未手配*")-COUNTIF(R6:R18,"*要確認*")-COUNTIF(R6:R18,"*NRT着*")-COUNTIF(R6:R18,"*HND着*")-COUNTIF(R6:R18,"*KIX着*")-COUNTIF(R6:R18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="S19" s="46">
         <f>COUNTA(S6:S18)-COUNTIF(S6:S18,"*未手配*")-COUNTIF(S6:S18,"*要確認*")-COUNTIF(S6:S18,"*NRT着*")-COUNTIF(S6:S18,"*HND着*")-COUNTIF(S6:S18,"*KIX着*")-COUNTIF(S6:S18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="107">
@@ -7433,75 +7433,75 @@
       </c>
       <c r="B20" s="47">
         <f>COUNTA(B17:B18)-COUNTIF(B17:B18,"*未手配*")-COUNTIF(B17:B18,"*要確認*")-COUNTIF(B17:B18,"*NRT着*")-COUNTIF(B17:B18,"*HND着*")-COUNTIF(B17:B18,"*KIX着*")-COUNTIF(B17:B18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C20" s="47">
         <f>COUNTA(C17:C18)-COUNTIF(C17:C18,"*未手配*")-COUNTIF(C17:C18,"*要確認*")-COUNTIF(C17:C18,"*NRT着*")-COUNTIF(C17:C18,"*HND着*")-COUNTIF(C17:C18,"*KIX着*")-COUNTIF(C17:C18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D20" s="47">
         <f>COUNTA(D17:D18)-COUNTIF(D17:D18,"*未手配*")-COUNTIF(D17:D18,"*要確認*")-COUNTIF(D17:D18,"*NRT着*")-COUNTIF(D17:D18,"*HND着*")-COUNTIF(D17:D18,"*KIX着*")-COUNTIF(D17:D18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E20" s="47">
         <f>COUNTA(E17:E18)-COUNTIF(E17:E18,"*未手配*")-COUNTIF(E17:E18,"*要確認*")-COUNTIF(E17:E18,"*NRT着*")-COUNTIF(E17:E18,"*HND着*")-COUNTIF(E17:E18,"*KIX着*")-COUNTIF(E17:E18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F20" s="47">
         <f>COUNTA(F17:F18)-COUNTIF(F17:F18,"*未手配*")-COUNTIF(F17:F18,"*要確認*")-COUNTIF(F17:F18,"*NRT着*")-COUNTIF(F17:F18,"*HND着*")-COUNTIF(F17:F18,"*KIX着*")-COUNTIF(F17:F18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="G20" s="47">
         <f>COUNTA(G17:G18)-COUNTIF(G17:G18,"*未手配*")-COUNTIF(G17:G18,"*要確認*")-COUNTIF(G17:G18,"*NRT着*")-COUNTIF(G17:G18,"*HND着*")-COUNTIF(G17:G18,"*KIX着*")-COUNTIF(G17:G18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="H20" s="47">
         <f>COUNTA(H17:H18)-COUNTIF(H17:H18,"*未手配*")-COUNTIF(H17:H18,"*要確認*")-COUNTIF(H17:H18,"*NRT着*")-COUNTIF(H17:H18,"*HND着*")-COUNTIF(H17:H18,"*KIX着*")-COUNTIF(H17:H18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I20" s="47">
         <f>COUNTA(I17:I18)-COUNTIF(I17:I18,"*未手配*")-COUNTIF(I17:I18,"*要確認*")-COUNTIF(I17:I18,"*NRT着*")-COUNTIF(I17:I18,"*HND着*")-COUNTIF(I17:I18,"*KIX着*")-COUNTIF(I17:I18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J20" s="47">
         <f>COUNTA(J17:J18)-COUNTIF(J17:J18,"*未手配*")-COUNTIF(J17:J18,"*要確認*")-COUNTIF(J17:J18,"*NRT着*")-COUNTIF(J17:J18,"*HND着*")-COUNTIF(J17:J18,"*KIX着*")-COUNTIF(J17:J18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K20" s="47">
         <f>COUNTA(K17:K18)-COUNTIF(K17:K18,"*未手配*")-COUNTIF(K17:K18,"*要確認*")-COUNTIF(K17:K18,"*NRT着*")-COUNTIF(K17:K18,"*HND着*")-COUNTIF(K17:K18,"*KIX着*")-COUNTIF(K17:K18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="L20" s="47">
         <f>COUNTA(L17:L18)-COUNTIF(L17:L18,"*未手配*")-COUNTIF(L17:L18,"*要確認*")-COUNTIF(L17:L18,"*NRT着*")-COUNTIF(L17:L18,"*HND着*")-COUNTIF(L17:L18,"*KIX着*")-COUNTIF(L17:L18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="M20" s="47">
         <f>COUNTA(M17:M18)-COUNTIF(M17:M18,"*未手配*")-COUNTIF(M17:M18,"*要確認*")-COUNTIF(M17:M18,"*NRT着*")-COUNTIF(M17:M18,"*HND着*")-COUNTIF(M17:M18,"*KIX着*")-COUNTIF(M17:M18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="N20" s="47">
         <f>COUNTA(N17:N18)-COUNTIF(N17:N18,"*未手配*")-COUNTIF(N17:N18,"*要確認*")-COUNTIF(N17:N18,"*NRT着*")-COUNTIF(N17:N18,"*HND着*")-COUNTIF(N17:N18,"*KIX着*")-COUNTIF(N17:N18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="O20" s="47">
         <f>COUNTA(O17:O18)-COUNTIF(O17:O18,"*未手配*")-COUNTIF(O17:O18,"*要確認*")-COUNTIF(O17:O18,"*NRT着*")-COUNTIF(O17:O18,"*HND着*")-COUNTIF(O17:O18,"*KIX着*")-COUNTIF(O17:O18,"*GVA着*")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P20" s="47">
         <f>COUNTA(P17:P18)-COUNTIF(P17:P18,"*未手配*")-COUNTIF(P17:P18,"*要確認*")-COUNTIF(P17:P18,"*NRT着*")-COUNTIF(P17:P18,"*HND着*")-COUNTIF(P17:P18,"*KIX着*")-COUNTIF(P17:P18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q20" s="47">
         <f>COUNTA(Q17:Q18)-COUNTIF(Q17:Q18,"*未手配*")-COUNTIF(Q17:Q18,"*要確認*")-COUNTIF(Q17:Q18,"*NRT着*")-COUNTIF(Q17:Q18,"*HND着*")-COUNTIF(Q17:Q18,"*KIX着*")-COUNTIF(Q17:Q18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R20" s="47">
         <f>COUNTA(R17:R18)-COUNTIF(R17:R18,"*未手配*")-COUNTIF(R17:R18,"*要確認*")-COUNTIF(R17:R18,"*NRT着*")-COUNTIF(R17:R18,"*HND着*")-COUNTIF(R17:R18,"*KIX着*")-COUNTIF(R17:R18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S20" s="47">
         <f>COUNTA(S17:S18)-COUNTIF(S17:S18,"*未手配*")-COUNTIF(S17:S18,"*要確認*")-COUNTIF(S17:S18,"*NRT着*")-COUNTIF(S17:S18,"*HND着*")-COUNTIF(S17:S18,"*KIX着*")-COUNTIF(S17:S18,"*GVA着*")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1" s="107">
@@ -7526,9 +7526,9 @@
       </c>
     </row>
     <row r="24" ht="39.75" customHeight="1" s="107">
-      <c r="A24" s="49">
+      <c r="A24" s="49" t="str">
         <f>人員一覧・判定!B18</f>
-        <v/>
+        <v>中村</v>
       </c>
       <c r="B24" s="29" t="n"/>
       <c r="C24" s="29" t="n"/>
@@ -7590,9 +7590,9 @@
       <c r="S24" s="29" t="n"/>
     </row>
     <row r="25" ht="39.75" customHeight="1" s="107">
-      <c r="A25" s="49">
+      <c r="A25" s="49" t="str">
         <f>人員一覧・判定!B19</f>
-        <v/>
+        <v>山口</v>
       </c>
       <c r="B25" s="29" t="n"/>
       <c r="C25" s="29" t="n"/>
@@ -7646,9 +7646,9 @@
       <c r="S25" s="29" t="n"/>
     </row>
     <row r="26" ht="39.75" customHeight="1" s="107">
-      <c r="A26" s="49">
+      <c r="A26" s="49" t="str">
         <f>人員一覧・判定!B21</f>
-        <v/>
+        <v>寺坂　佳津子</v>
       </c>
       <c r="B26" s="29" t="n"/>
       <c r="C26" s="29" t="n"/>
@@ -7686,9 +7686,9 @@
       <c r="S26" s="29" t="n"/>
     </row>
     <row r="27" ht="39.75" customHeight="1" s="107">
-      <c r="A27" s="49">
+      <c r="A27" s="49" t="str">
         <f>人員一覧・判定!B20</f>
-        <v/>
+        <v>伊達 孝</v>
       </c>
       <c r="B27" s="29" t="n"/>
       <c r="C27" s="29" t="n"/>
@@ -7953,9 +7953,9 @@
       <c r="AC5" s="102" t="n"/>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="107">
-      <c r="A6" s="40">
+      <c r="A6" s="40" t="str">
         <f>人員一覧・判定!B5</f>
-        <v/>
+        <v>三浦 房紀</v>
       </c>
       <c r="H6" s="154" t="inlineStr">
         <is>
@@ -7977,9 +7977,9 @@
       <c r="AD6" s="95" t="n"/>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="107">
-      <c r="A7" s="40">
+      <c r="A7" s="40" t="str">
         <f>人員一覧・判定!B6</f>
-        <v/>
+        <v>北本 政行</v>
       </c>
       <c r="H7" s="154" t="inlineStr">
         <is>
@@ -8001,9 +8001,9 @@
       <c r="AD7" s="95" t="n"/>
     </row>
     <row r="8" ht="21.75" customHeight="1" s="107">
-      <c r="A8" s="40">
+      <c r="A8" s="40" t="str">
         <f>人員一覧・判定!B7</f>
-        <v/>
+        <v>宮木 一寛</v>
       </c>
       <c r="F8" s="155" t="inlineStr">
         <is>
@@ -8029,9 +8029,9 @@
       <c r="AD8" s="95" t="n"/>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="107">
-      <c r="A9" s="40">
+      <c r="A9" s="40" t="str">
         <f>人員一覧・判定!B8</f>
-        <v/>
+        <v>児玉 美樹</v>
       </c>
       <c r="F9" s="154" t="inlineStr">
         <is>
@@ -8064,9 +8064,9 @@
       <c r="AD9" s="95" t="n"/>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="107">
-      <c r="A10" s="40">
+      <c r="A10" s="40" t="str">
         <f>人員一覧・判定!B9</f>
-        <v/>
+        <v>荒木田 勝</v>
       </c>
       <c r="F10" s="154" t="inlineStr">
         <is>
@@ -8109,9 +8109,9 @@
       <c r="AE10" s="95" t="n"/>
     </row>
     <row r="11" ht="21.75" customHeight="1" s="107">
-      <c r="A11" s="40">
+      <c r="A11" s="40" t="str">
         <f>人員一覧・判定!B10</f>
-        <v/>
+        <v>吉田 真紀</v>
       </c>
       <c r="F11" s="154" t="inlineStr">
         <is>
@@ -8144,9 +8144,9 @@
       <c r="AD11" s="95" t="n"/>
     </row>
     <row r="12" ht="21.75" customHeight="1" s="107">
-      <c r="A12" s="40">
+      <c r="A12" s="40" t="str">
         <f>人員一覧・判定!B11</f>
-        <v/>
+        <v>藤中 純子</v>
       </c>
       <c r="D12" s="159" t="inlineStr">
         <is>
@@ -8187,9 +8187,9 @@
       <c r="AD12" s="95" t="n"/>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="107">
-      <c r="A13" s="40">
+      <c r="A13" s="40" t="str">
         <f>人員一覧・判定!B12</f>
-        <v/>
+        <v>田中 智美</v>
       </c>
       <c r="D13" s="159" t="inlineStr">
         <is>
@@ -8230,9 +8230,9 @@
       <c r="AD13" s="95" t="n"/>
     </row>
     <row r="14" ht="21.75" customHeight="1" s="107">
-      <c r="A14" s="40">
+      <c r="A14" s="40" t="str">
         <f>人員一覧・判定!B13</f>
-        <v/>
+        <v>池田　誠</v>
       </c>
       <c r="F14" s="156" t="inlineStr">
         <is>
@@ -8268,9 +8268,9 @@
       <c r="AD14" s="95" t="n"/>
     </row>
     <row r="15" ht="24.75" customHeight="1" s="107">
-      <c r="A15" s="58">
+      <c r="A15" s="58" t="str">
         <f>人員一覧・判定!C14</f>
-        <v/>
+        <v>Gerald Ejem Potutan</v>
       </c>
       <c r="F15" s="154" t="inlineStr">
         <is>
@@ -8311,9 +8311,9 @@
       <c r="AD15" s="95" t="n"/>
     </row>
     <row r="16" ht="21" customHeight="1" s="107">
-      <c r="A16" s="40">
+      <c r="A16" s="40" t="str">
         <f>人員一覧・判定!C15</f>
-        <v/>
+        <v>Mizan Bisri</v>
       </c>
       <c r="F16" s="154" t="inlineStr">
         <is>
@@ -8356,9 +8356,9 @@
       <c r="AD16" s="95" t="n"/>
     </row>
     <row r="17" ht="21.75" customHeight="1" s="107">
-      <c r="A17" s="40">
+      <c r="A17" s="40" t="str">
         <f>人員一覧・判定!B16</f>
-        <v/>
+        <v>藤本 絢子</v>
       </c>
       <c r="F17" s="154" t="inlineStr">
         <is>
@@ -8401,9 +8401,9 @@
       <c r="AD17" s="95" t="n"/>
     </row>
     <row r="18" ht="21.75" customHeight="1" s="107">
-      <c r="A18" s="40">
+      <c r="A18" s="40" t="str">
         <f>人員一覧・判定!B17</f>
-        <v/>
+        <v>塩見 有美</v>
       </c>
       <c r="F18" s="158" t="inlineStr">
         <is>
@@ -8449,131 +8449,131 @@
       </c>
       <c r="B19" s="59">
         <f>COUNTA(B5:B18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C19" s="59">
         <f>COUNTA(C5:C18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="59">
         <f>COUNTA(D5:D18)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E19" s="59">
         <f>COUNTA(E5:E18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F19" s="59">
         <f>COUNTA(F5:F18)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="G19" s="59">
         <f>COUNTA(G5:G18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H19" s="59">
         <f>COUNTA(H5:H18)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I19" s="59">
         <f>COUNTA(I5:I18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J19" s="59">
         <f>COUNTA(J5:J18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K19" s="59">
         <f>COUNTA(K5:K18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L19" s="59">
         <f>COUNTA(L5:L18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M19" s="59">
         <f>COUNTA(M5:M18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N19" s="59">
         <f>COUNTA(N5:N18)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="O19" s="59">
         <f>COUNTA(O5:O18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P19" s="59">
         <f>COUNTA(P5:P18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q19" s="59">
         <f>COUNTA(Q5:Q18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R19" s="59">
         <f>COUNTA(R5:R18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S19" s="59">
         <f>COUNTA(S5:S18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T19" s="59">
         <f>COUNTA(T5:T18)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="U19" s="59">
         <f>COUNTA(U5:U18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V19" s="59">
         <f>COUNTA(V5:V18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="W19" s="59">
         <f>COUNTA(W5:W18)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="X19" s="59">
         <f>COUNTA(X5:X18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y19" s="59">
         <f>COUNTA(Y5:Y18)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="Z19" s="59">
         <f>COUNTA(Z5:Z18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA19" s="59">
         <f>COUNTA(AA5:AA18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB19" s="59">
         <f>COUNTA(AB5:AB18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC19" s="59">
         <f>COUNTA(AC5:AC18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD19" s="59">
         <f>COUNTA(AD5:AD18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AE19" s="59">
         <f>COUNTA(AE5:AE18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF19" s="59">
         <f>COUNTA(AF5:AF18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG19" s="59">
         <f>COUNTA(AG5:AG18)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="107">
@@ -8600,9 +8600,9 @@
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1" s="107">
-      <c r="A24" s="49">
+      <c r="A24" s="49" t="str">
         <f>人員一覧・判定!B18</f>
-        <v/>
+        <v>中村</v>
       </c>
       <c r="F24" s="162" t="inlineStr">
         <is>
@@ -8626,9 +8626,9 @@
       <c r="S24" s="95" t="n"/>
     </row>
     <row r="25" ht="21.75" customHeight="1" s="107">
-      <c r="A25" s="49">
+      <c r="A25" s="49" t="str">
         <f>人員一覧・判定!B19</f>
-        <v/>
+        <v>山口</v>
       </c>
       <c r="F25" s="164" t="inlineStr">
         <is>
@@ -8652,9 +8652,9 @@
       <c r="S25" s="95" t="n"/>
     </row>
     <row r="26" ht="21.75" customHeight="1" s="107">
-      <c r="A26" s="49">
+      <c r="A26" s="49" t="str">
         <f>人員一覧・判定!B21</f>
-        <v/>
+        <v>寺坂　佳津子</v>
       </c>
       <c r="N26" s="165" t="inlineStr">
         <is>
@@ -8668,9 +8668,9 @@
       <c r="S26" s="95" t="n"/>
     </row>
     <row r="27" ht="21.75" customHeight="1" s="107">
-      <c r="A27" s="49">
+      <c r="A27" s="49" t="str">
         <f>人員一覧・判定!B20</f>
-        <v/>
+        <v>伊達 孝</v>
       </c>
       <c r="N27" s="166" t="inlineStr">
         <is>
@@ -8959,9 +8959,9 @@
       <c r="AC5" s="97" t="n"/>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="107">
-      <c r="A6" s="40">
+      <c r="A6" s="40" t="str">
         <f>人員一覧・判定!B5</f>
-        <v/>
+        <v>三浦 房紀</v>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
@@ -9004,9 +9004,9 @@
       <c r="AC6" s="95" t="n"/>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="107">
-      <c r="A7" s="40">
+      <c r="A7" s="40" t="str">
         <f>人員一覧・判定!B6</f>
-        <v/>
+        <v>北本 政行</v>
       </c>
       <c r="G7" s="168" t="inlineStr">
         <is>
@@ -9045,9 +9045,9 @@
       <c r="AC7" s="95" t="n"/>
     </row>
     <row r="8" ht="21.75" customHeight="1" s="107">
-      <c r="A8" s="40">
+      <c r="A8" s="40" t="str">
         <f>人員一覧・判定!B7</f>
-        <v/>
+        <v>宮木 一寛</v>
       </c>
       <c r="F8" s="155" t="inlineStr">
         <is>
@@ -9087,9 +9087,9 @@
       <c r="AC8" s="95" t="n"/>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="107">
-      <c r="A9" s="40">
+      <c r="A9" s="40" t="str">
         <f>人員一覧・判定!B8</f>
-        <v/>
+        <v>児玉 美樹</v>
       </c>
       <c r="C9" s="171" t="inlineStr">
         <is>
@@ -9137,9 +9137,9 @@
       <c r="AC9" s="95" t="n"/>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="107">
-      <c r="A10" s="40">
+      <c r="A10" s="40" t="str">
         <f>人員一覧・判定!B9</f>
-        <v/>
+        <v>荒木田 勝</v>
       </c>
       <c r="C10" s="172" t="inlineStr">
         <is>
@@ -9190,9 +9190,9 @@
       <c r="AC10" s="95" t="n"/>
     </row>
     <row r="11" ht="21.75" customHeight="1" s="107">
-      <c r="A11" s="40">
+      <c r="A11" s="40" t="str">
         <f>人員一覧・判定!B10</f>
-        <v/>
+        <v>吉田 真紀</v>
       </c>
       <c r="D11" s="173" t="inlineStr">
         <is>
@@ -9239,9 +9239,9 @@
       <c r="AC11" s="95" t="n"/>
     </row>
     <row r="12" ht="21.75" customHeight="1" s="107">
-      <c r="A12" s="40">
+      <c r="A12" s="40" t="str">
         <f>人員一覧・判定!B11</f>
-        <v/>
+        <v>藤中 純子</v>
       </c>
       <c r="C12" s="174" t="inlineStr">
         <is>
@@ -9290,9 +9290,9 @@
       <c r="AC12" s="95" t="n"/>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="107">
-      <c r="A13" s="40">
+      <c r="A13" s="40" t="str">
         <f>人員一覧・判定!B12</f>
-        <v/>
+        <v>田中 智美</v>
       </c>
       <c r="C13" s="174" t="inlineStr">
         <is>
@@ -9342,9 +9342,9 @@
       <c r="AC13" s="95" t="n"/>
     </row>
     <row r="14" ht="21.75" customHeight="1" s="107">
-      <c r="A14" s="40">
+      <c r="A14" s="40" t="str">
         <f>人員一覧・判定!B13</f>
-        <v/>
+        <v>池田　誠</v>
       </c>
       <c r="C14" s="171" t="inlineStr">
         <is>
@@ -9391,9 +9391,9 @@
       <c r="AC14" s="95" t="n"/>
     </row>
     <row r="15" ht="21.75" customHeight="1" s="107">
-      <c r="A15" s="58">
+      <c r="A15" s="58" t="str">
         <f>人員一覧・判定!C14</f>
-        <v/>
+        <v>Gerald Ejem Potutan</v>
       </c>
       <c r="C15" s="176" t="inlineStr">
         <is>
@@ -9447,9 +9447,9 @@
       <c r="AF15" s="95" t="n"/>
     </row>
     <row r="16" ht="21.75" customHeight="1" s="107">
-      <c r="A16" s="40">
+      <c r="A16" s="40" t="str">
         <f>人員一覧・判定!C15</f>
-        <v/>
+        <v>Mizan Bisri</v>
       </c>
       <c r="C16" s="174" t="inlineStr">
         <is>
@@ -9496,9 +9496,9 @@
       <c r="AC16" s="95" t="n"/>
     </row>
     <row r="17" ht="21.75" customHeight="1" s="107">
-      <c r="A17" s="40">
+      <c r="A17" s="40" t="str">
         <f>人員一覧・判定!B16</f>
-        <v/>
+        <v>藤本 絢子</v>
       </c>
       <c r="C17" s="171" t="inlineStr">
         <is>
@@ -9541,9 +9541,9 @@
       <c r="AC17" s="95" t="n"/>
     </row>
     <row r="18" ht="21.75" customHeight="1" s="107">
-      <c r="A18" s="40">
+      <c r="A18" s="40" t="str">
         <f>人員一覧・判定!B17</f>
-        <v/>
+        <v>塩見 有美</v>
       </c>
       <c r="C18" s="174" t="inlineStr">
         <is>
@@ -9597,131 +9597,131 @@
       </c>
       <c r="B19" s="59">
         <f>COUNTA(B5:B18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C19" s="59">
         <f>COUNTA(C5:C18)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="D19" s="59">
         <f>COUNTA(D5:D18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="E19" s="59">
         <f>COUNTA(E5:E18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F19" s="59">
         <f>COUNTA(F5:F18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G19" s="59">
         <f>COUNTA(G5:G18)</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="H19" s="59">
         <f>COUNTA(H5:H18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I19" s="59">
         <f>COUNTA(I5:I18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J19" s="59">
         <f>COUNTA(J5:J18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K19" s="59">
         <f>COUNTA(K5:K18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L19" s="59">
         <f>COUNTA(L5:L18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M19" s="59">
         <f>COUNTA(M5:M18)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="N19" s="59">
         <f>COUNTA(N5:N18)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="O19" s="59">
         <f>COUNTA(O5:O18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P19" s="59">
         <f>COUNTA(P5:P18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q19" s="59">
         <f>COUNTA(Q5:Q18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R19" s="59">
         <f>COUNTA(R5:R18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S19" s="59">
         <f>COUNTA(S5:S18)</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="T19" s="59">
         <f>COUNTA(T5:T18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U19" s="59">
         <f>COUNTA(U5:U18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V19" s="59">
         <f>COUNTA(V5:V18)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="W19" s="59">
         <f>COUNTA(W5:W18)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="X19" s="59">
         <f>COUNTA(X5:X18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y19" s="59">
         <f>COUNTA(Y5:Y18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z19" s="59">
         <f>COUNTA(Z5:Z18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA19" s="59">
         <f>COUNTA(AA5:AA18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB19" s="59">
         <f>COUNTA(AB5:AB18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC19" s="59">
         <f>COUNTA(AC5:AC18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD19" s="59">
         <f>COUNTA(AD5:AD18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AE19" s="59">
         <f>COUNTA(AE5:AE18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF19" s="59">
         <f>COUNTA(AF5:AF18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG19" s="59">
         <f>COUNTA(AG5:AG18)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="107">
@@ -9757,9 +9757,9 @@
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1" s="107">
-      <c r="A24" s="49">
+      <c r="A24" s="49" t="str">
         <f>人員一覧・判定!B18</f>
-        <v/>
+        <v>中村</v>
       </c>
       <c r="D24" s="181" t="inlineStr">
         <is>
@@ -9786,9 +9786,9 @@
       <c r="T24" s="95" t="n"/>
     </row>
     <row r="25" ht="21.75" customHeight="1" s="107">
-      <c r="A25" s="49">
+      <c r="A25" s="49" t="str">
         <f>人員一覧・判定!B19</f>
-        <v/>
+        <v>山口</v>
       </c>
       <c r="D25" s="161" t="inlineStr">
         <is>
@@ -9815,9 +9815,9 @@
       <c r="T25" s="95" t="n"/>
     </row>
     <row r="26" ht="21.75" customHeight="1" s="107">
-      <c r="A26" s="49">
+      <c r="A26" s="49" t="str">
         <f>人員一覧・判定!B21</f>
-        <v/>
+        <v>寺坂　佳津子</v>
       </c>
       <c r="M26" s="165" t="inlineStr">
         <is>
@@ -9833,9 +9833,9 @@
       <c r="T26" s="95" t="n"/>
     </row>
     <row r="27" ht="21.75" customHeight="1" s="107">
-      <c r="A27" s="49">
+      <c r="A27" s="49" t="str">
         <f>人員一覧・判定!B20</f>
-        <v/>
+        <v>伊達 孝</v>
       </c>
       <c r="D27" s="183" t="inlineStr">
         <is>
@@ -10155,9 +10155,9 @@
       <c r="AD5" s="97" t="n"/>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="107">
-      <c r="A6" s="40">
+      <c r="A6" s="40" t="str">
         <f>人員一覧・判定!B5</f>
-        <v/>
+        <v>三浦 房紀</v>
       </c>
       <c r="G6" s="169" t="inlineStr">
         <is>
@@ -10197,9 +10197,9 @@
       <c r="AD6" s="95" t="n"/>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="107">
-      <c r="A7" s="40">
+      <c r="A7" s="40" t="str">
         <f>人員一覧・判定!B6</f>
-        <v/>
+        <v>北本 政行</v>
       </c>
       <c r="G7" s="169" t="inlineStr">
         <is>
@@ -10239,9 +10239,9 @@
       <c r="AD7" s="95" t="n"/>
     </row>
     <row r="8" ht="21.75" customHeight="1" s="107">
-      <c r="A8" s="40">
+      <c r="A8" s="40" t="str">
         <f>人員一覧・判定!B7</f>
-        <v/>
+        <v>宮木 一寛</v>
       </c>
       <c r="G8" s="169" t="inlineStr">
         <is>
@@ -10281,9 +10281,9 @@
       <c r="AD8" s="95" t="n"/>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="107">
-      <c r="A9" s="40">
+      <c r="A9" s="40" t="str">
         <f>人員一覧・判定!B8</f>
-        <v/>
+        <v>児玉 美樹</v>
       </c>
       <c r="D9" s="156" t="inlineStr">
         <is>
@@ -10326,9 +10326,9 @@
       <c r="AD9" s="95" t="n"/>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="107">
-      <c r="A10" s="40">
+      <c r="A10" s="40" t="str">
         <f>人員一覧・判定!B9</f>
-        <v/>
+        <v>荒木田 勝</v>
       </c>
       <c r="D10" s="188" t="inlineStr">
         <is>
@@ -10376,9 +10376,9 @@
       <c r="AD10" s="95" t="n"/>
     </row>
     <row r="11" ht="21.75" customHeight="1" s="107">
-      <c r="A11" s="40">
+      <c r="A11" s="40" t="str">
         <f>人員一覧・判定!B10</f>
-        <v/>
+        <v>吉田 真紀</v>
       </c>
       <c r="D11" s="178" t="inlineStr">
         <is>
@@ -10428,9 +10428,9 @@
       <c r="AD11" s="95" t="n"/>
     </row>
     <row r="12" ht="21.75" customHeight="1" s="107">
-      <c r="A12" s="40">
+      <c r="A12" s="40" t="str">
         <f>人員一覧・判定!B11</f>
-        <v/>
+        <v>藤中 純子</v>
       </c>
       <c r="D12" s="158" t="inlineStr">
         <is>
@@ -10469,9 +10469,9 @@
       <c r="AD12" s="95" t="n"/>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="107">
-      <c r="A13" s="40">
+      <c r="A13" s="40" t="str">
         <f>人員一覧・判定!B12</f>
-        <v/>
+        <v>田中 智美</v>
       </c>
       <c r="D13" s="158" t="inlineStr">
         <is>
@@ -10517,9 +10517,9 @@
       <c r="AD13" s="95" t="n"/>
     </row>
     <row r="14" ht="21.75" customHeight="1" s="107">
-      <c r="A14" s="40">
+      <c r="A14" s="40" t="str">
         <f>人員一覧・判定!B13</f>
-        <v/>
+        <v>池田　誠</v>
       </c>
       <c r="D14" s="190" t="inlineStr">
         <is>
@@ -10561,9 +10561,9 @@
       <c r="AD14" s="95" t="n"/>
     </row>
     <row r="15" ht="21.75" customHeight="1" s="107">
-      <c r="A15" s="58">
+      <c r="A15" s="58" t="str">
         <f>人員一覧・判定!C14</f>
-        <v/>
+        <v>Gerald Ejem Potutan</v>
       </c>
       <c r="D15" s="191" t="inlineStr">
         <is>
@@ -10610,9 +10610,9 @@
       <c r="AD15" s="95" t="n"/>
     </row>
     <row r="16" ht="21.75" customHeight="1" s="107">
-      <c r="A16" s="40">
+      <c r="A16" s="40" t="str">
         <f>人員一覧・判定!C15</f>
-        <v/>
+        <v>Mizan Bisri</v>
       </c>
       <c r="D16" s="171" t="inlineStr">
         <is>
@@ -10654,9 +10654,9 @@
       <c r="AD16" s="95" t="n"/>
     </row>
     <row r="17" ht="21.75" customHeight="1" s="107">
-      <c r="A17" s="40">
+      <c r="A17" s="40" t="str">
         <f>人員一覧・判定!B16</f>
-        <v/>
+        <v>藤本 絢子</v>
       </c>
       <c r="D17" s="156" t="inlineStr">
         <is>
@@ -10699,9 +10699,9 @@
       <c r="AD17" s="95" t="n"/>
     </row>
     <row r="18" ht="21.75" customHeight="1" s="107">
-      <c r="A18" s="40">
+      <c r="A18" s="40" t="str">
         <f>人員一覧・判定!B17</f>
-        <v/>
+        <v>塩見 有美</v>
       </c>
       <c r="D18" s="178" t="inlineStr">
         <is>
@@ -10757,131 +10757,131 @@
       </c>
       <c r="B19" s="59">
         <f>COUNTA(B5:B18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C19" s="59">
         <f>COUNTA(C5:C18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="59">
         <f>COUNTA(D5:D18)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="E19" s="59">
         <f>COUNTA(E5:E18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F19" s="59">
         <f>COUNTA(F5:F18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G19" s="59">
         <f>COUNTA(G5:G18)</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="H19" s="59">
         <f>COUNTA(H5:H18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I19" s="59">
         <f>COUNTA(I5:I18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J19" s="59">
         <f>COUNTA(J5:J18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K19" s="59">
         <f>COUNTA(K5:K18)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="L19" s="59">
         <f>COUNTA(L5:L18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M19" s="59">
         <f>COUNTA(M5:M18)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="N19" s="59">
         <f>COUNTA(N5:N18)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="O19" s="59">
         <f>COUNTA(O5:O18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P19" s="59">
         <f>COUNTA(P5:P18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q19" s="59">
         <f>COUNTA(Q5:Q18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R19" s="59">
         <f>COUNTA(R5:R18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S19" s="59">
         <f>COUNTA(S5:S18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T19" s="59">
         <f>COUNTA(T5:T18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U19" s="59">
         <f>COUNTA(U5:U18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V19" s="59">
         <f>COUNTA(V5:V18)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="W19" s="59">
         <f>COUNTA(W5:W18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="X19" s="59">
         <f>COUNTA(X5:X18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y19" s="59">
         <f>COUNTA(Y5:Y18)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="Z19" s="59">
         <f>COUNTA(Z5:Z18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA19" s="59">
         <f>COUNTA(AA5:AA18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB19" s="59">
         <f>COUNTA(AB5:AB18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC19" s="59">
         <f>COUNTA(AC5:AC18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD19" s="59">
         <f>COUNTA(AD5:AD18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AE19" s="59">
         <f>COUNTA(AE5:AE18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF19" s="59">
         <f>COUNTA(AF5:AF18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG19" s="59">
         <f>COUNTA(AG5:AG18)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="107">
@@ -10914,9 +10914,9 @@
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1" s="107">
-      <c r="A24" s="49">
+      <c r="A24" s="49" t="str">
         <f>人員一覧・判定!B18</f>
-        <v/>
+        <v>中村</v>
       </c>
       <c r="D24" s="162" t="inlineStr">
         <is>
@@ -10942,9 +10942,9 @@
       <c r="O24" s="95" t="n"/>
     </row>
     <row r="25" ht="21.75" customHeight="1" s="107">
-      <c r="A25" s="49">
+      <c r="A25" s="49" t="str">
         <f>人員一覧・判定!B19</f>
-        <v/>
+        <v>山口</v>
       </c>
       <c r="D25" s="161" t="inlineStr">
         <is>
@@ -10974,9 +10974,9 @@
       <c r="S25" s="95" t="n"/>
     </row>
     <row r="26" ht="21.75" customHeight="1" s="107">
-      <c r="A26" s="49">
+      <c r="A26" s="49" t="str">
         <f>人員一覧・判定!B21</f>
-        <v/>
+        <v>寺坂　佳津子</v>
       </c>
       <c r="G26" s="194" t="inlineStr">
         <is>
@@ -10989,9 +10989,9 @@
       <c r="K26" s="95" t="n"/>
     </row>
     <row r="27" ht="21.75" customHeight="1" s="107">
-      <c r="A27" s="49">
+      <c r="A27" s="49" t="str">
         <f>人員一覧・判定!B20</f>
-        <v/>
+        <v>伊達 孝</v>
       </c>
       <c r="D27" s="166" t="inlineStr">
         <is>
@@ -11287,9 +11287,9 @@
       <c r="AF5" s="102" t="n"/>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="107">
-      <c r="A6" s="40">
+      <c r="A6" s="40" t="str">
         <f>人員一覧・判定!B5</f>
-        <v/>
+        <v>三浦 房紀</v>
       </c>
       <c r="F6" s="169" t="inlineStr">
         <is>
@@ -11320,9 +11320,9 @@
       <c r="AF6" s="95" t="n"/>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="107">
-      <c r="A7" s="40">
+      <c r="A7" s="40" t="str">
         <f>人員一覧・判定!B6</f>
-        <v/>
+        <v>北本 政行</v>
       </c>
       <c r="F7" s="169" t="inlineStr">
         <is>
@@ -11354,9 +11354,9 @@
       <c r="AF7" s="95" t="n"/>
     </row>
     <row r="8" ht="21.75" customHeight="1" s="107">
-      <c r="A8" s="40">
+      <c r="A8" s="40" t="str">
         <f>人員一覧・判定!B7</f>
-        <v/>
+        <v>宮木 一寛</v>
       </c>
       <c r="F8" s="169" t="inlineStr">
         <is>
@@ -11388,9 +11388,9 @@
       <c r="Y8" s="95" t="n"/>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="107">
-      <c r="A9" s="40">
+      <c r="A9" s="40" t="str">
         <f>人員一覧・判定!B8</f>
-        <v/>
+        <v>児玉 美樹</v>
       </c>
       <c r="F9" s="169" t="inlineStr">
         <is>
@@ -11424,9 +11424,9 @@
       <c r="AA9" s="95" t="n"/>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="107">
-      <c r="A10" s="40">
+      <c r="A10" s="40" t="str">
         <f>人員一覧・判定!B9</f>
-        <v/>
+        <v>荒木田 勝</v>
       </c>
       <c r="F10" s="169" t="inlineStr">
         <is>
@@ -11468,9 +11468,9 @@
       <c r="AF10" s="95" t="n"/>
     </row>
     <row r="11" ht="21.75" customHeight="1" s="107">
-      <c r="A11" s="40">
+      <c r="A11" s="40" t="str">
         <f>人員一覧・判定!B10</f>
-        <v/>
+        <v>吉田 真紀</v>
       </c>
       <c r="D11" s="197" t="inlineStr">
         <is>
@@ -11517,9 +11517,9 @@
       <c r="AF11" s="95" t="n"/>
     </row>
     <row r="12" ht="21.75" customHeight="1" s="107">
-      <c r="A12" s="40">
+      <c r="A12" s="40" t="str">
         <f>人員一覧・判定!B11</f>
-        <v/>
+        <v>藤中 純子</v>
       </c>
       <c r="F12" s="158" t="inlineStr">
         <is>
@@ -11555,9 +11555,9 @@
       <c r="AC12" s="95" t="n"/>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="107">
-      <c r="A13" s="40">
+      <c r="A13" s="40" t="str">
         <f>人員一覧・判定!B12</f>
-        <v/>
+        <v>田中 智美</v>
       </c>
       <c r="D13" s="197" t="inlineStr">
         <is>
@@ -11599,9 +11599,9 @@
       <c r="AC13" s="95" t="n"/>
     </row>
     <row r="14" ht="21.75" customHeight="1" s="107">
-      <c r="A14" s="40">
+      <c r="A14" s="40" t="str">
         <f>人員一覧・判定!B13</f>
-        <v/>
+        <v>池田　誠</v>
       </c>
       <c r="F14" s="169" t="inlineStr">
         <is>
@@ -11643,9 +11643,9 @@
       <c r="AF14" s="95" t="n"/>
     </row>
     <row r="15" ht="21.75" customHeight="1" s="107">
-      <c r="A15" s="58">
+      <c r="A15" s="58" t="str">
         <f>人員一覧・判定!C14</f>
-        <v/>
+        <v>Gerald Ejem Potutan</v>
       </c>
       <c r="F15" s="169" t="inlineStr">
         <is>
@@ -11675,9 +11675,9 @@
       <c r="AF15" s="95" t="n"/>
     </row>
     <row r="16" ht="21.75" customHeight="1" s="107">
-      <c r="A16" s="40">
+      <c r="A16" s="40" t="str">
         <f>人員一覧・判定!C15</f>
-        <v/>
+        <v>Mizan Bisri</v>
       </c>
       <c r="F16" s="169" t="inlineStr">
         <is>
@@ -11701,9 +11701,9 @@
       <c r="T16" s="95" t="n"/>
     </row>
     <row r="17" ht="21.75" customHeight="1" s="107">
-      <c r="A17" s="40">
+      <c r="A17" s="40" t="str">
         <f>人員一覧・判定!B16</f>
-        <v/>
+        <v>藤本 絢子</v>
       </c>
       <c r="F17" s="156" t="inlineStr">
         <is>
@@ -11737,9 +11737,9 @@
       <c r="AA17" s="95" t="n"/>
     </row>
     <row r="18" ht="21.75" customHeight="1" s="107">
-      <c r="A18" s="40">
+      <c r="A18" s="40" t="str">
         <f>人員一覧・判定!B17</f>
-        <v/>
+        <v>塩見 有美</v>
       </c>
       <c r="F18" s="179" t="inlineStr">
         <is>
@@ -11780,131 +11780,131 @@
       </c>
       <c r="B19" s="59">
         <f>COUNTA(B5:B18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C19" s="59">
         <f>COUNTA(C5:C18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="59">
         <f>COUNTA(D5:D18)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E19" s="59">
         <f>COUNTA(E5:E18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F19" s="59">
         <f>COUNTA(F5:F18)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="G19" s="59">
         <f>COUNTA(G5:G18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H19" s="59">
         <f>COUNTA(H5:H18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I19" s="59">
         <f>COUNTA(I5:I18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J19" s="59">
         <f>COUNTA(J5:J18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K19" s="59">
         <f>COUNTA(K5:K18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L19" s="59">
         <f>COUNTA(L5:L18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M19" s="59">
         <f>COUNTA(M5:M18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N19" s="59">
         <f>COUNTA(N5:N18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O19" s="59">
         <f>COUNTA(O5:O18)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="P19" s="59">
         <f>COUNTA(P5:P18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q19" s="59">
         <f>COUNTA(Q5:Q18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R19" s="59">
         <f>COUNTA(R5:R18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="S19" s="59">
         <f>COUNTA(S5:S18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T19" s="59">
         <f>COUNTA(T5:T18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U19" s="59">
         <f>COUNTA(U5:U18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V19" s="59">
         <f>COUNTA(V5:V18)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="W19" s="59">
         <f>COUNTA(W5:W18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="X19" s="59">
         <f>COUNTA(X5:X18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y19" s="59">
         <f>COUNTA(Y5:Y18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z19" s="59">
         <f>COUNTA(Z5:Z18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA19" s="59">
         <f>COUNTA(AA5:AA18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB19" s="59">
         <f>COUNTA(AB5:AB18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AC19" s="59">
         <f>COUNTA(AC5:AC18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AD19" s="59">
         <f>COUNTA(AD5:AD18)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AE19" s="59">
         <f>COUNTA(AE5:AE18)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="AF19" s="59">
         <f>COUNTA(AF5:AF18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG19" s="59">
         <f>COUNTA(AG5:AG18)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="107">
@@ -11927,9 +11927,9 @@
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1" s="107">
-      <c r="A24" s="49">
+      <c r="A24" s="49" t="str">
         <f>人員一覧・判定!B18</f>
-        <v/>
+        <v>中村</v>
       </c>
       <c r="F24" s="200" t="inlineStr">
         <is>
@@ -11943,9 +11943,9 @@
       <c r="K24" s="95" t="n"/>
     </row>
     <row r="25" ht="21.75" customHeight="1" s="107">
-      <c r="A25" s="49">
+      <c r="A25" s="49" t="str">
         <f>人員一覧・判定!B19</f>
-        <v/>
+        <v>山口</v>
       </c>
       <c r="F25" s="161" t="inlineStr">
         <is>
@@ -15415,7 +15415,7 @@
       </c>
       <c r="C72" s="79">
         <f>COUNTIF(I5:I64,"未協議")</f>
-        <v/>
+        <v>25</v>
       </c>
     </row>
     <row r="73">
@@ -15426,7 +15426,7 @@
       </c>
       <c r="C73" s="79">
         <f>COUNTIF(I5:I64,"協議中")</f>
-        <v/>
+        <v>29</v>
       </c>
     </row>
     <row r="74">
@@ -15437,7 +15437,7 @@
       </c>
       <c r="C74" s="79">
         <f>COUNTIF(I5:I64,"合意")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>